<commit_message>
Fix a transcription error in the content template's example rows
Verified the workbook by diffing every field of every one of its 11
worked-example rows against the actual shipped lesson files
(src/content/lessons/**/*.ts) programmatically, not just eyeballing it.
Found one real discrepancy: a curly apostrophe (') in the source vs. a
straight one (') in the row I'd retyped for Day 1's final speak prompt —
cosmetic, but wrong is wrong, so fixed it and confirmed a clean re-diff
(0 discrepancies across all 11 rows). Also fixed a missing wrap_text
alignment on the Instructions sheet's leftmost column.

Also verified separately: Skills Reference matches skills.json exactly
(49/49 rows), quest_type_ref's dropdown values match days.json's actual
quest_N_type casing (lowercase, not quest-types.json's display-cased
labels), data validation ranges cover all 51 data rows, and the file's
zip/xlsx structure is intact.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/supernova_content_template.xlsx
+++ b/docs/templates/supernova_content_template.xlsx
@@ -131,7 +131,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1202,7 +1204,7 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Last one — put it all together. Give a full introduction: your name, where you're from, what you do, and one interest.</t>
+          <t>Last one — put it all together. Give a full introduction: your name, where you’re from, what you do, and one interest.</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr"/>

</xml_diff>